<commit_message>
feat(frontend): resolve 'Name-<ID>' on booked-cell click via ID-first lookup
</commit_message>
<xml_diff>
--- a/api/data/Test.xlsx
+++ b/api/data/Test.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3438" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3438" uniqueCount="24">
   <si>
     <t>AM</t>
   </si>
@@ -66,6 +66,9 @@
   </si>
   <si>
     <t>Nisreen Dagher [SID:113602689684]</t>
+  </si>
+  <si>
+    <t>Dhwani Patel [SID:139582853530]</t>
   </si>
   <si>
     <t>Lab B</t>
@@ -910,10 +913,10 @@
         <v>16</v>
       </c>
       <c r="K7" s="7" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="L7" s="7" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="M7" s="7" t="s">
         <v>8</v>
@@ -2376,7 +2379,7 @@
     </row>
     <row r="41" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A41" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B41" s="14">
         <v>1</v>
@@ -2420,7 +2423,7 @@
     </row>
     <row r="42" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B42" s="14">
         <v>2</v>
@@ -2464,7 +2467,7 @@
     </row>
     <row r="43" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A43" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B43" s="14">
         <v>3</v>
@@ -2508,7 +2511,7 @@
     </row>
     <row r="44" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B44" s="14">
         <v>4</v>
@@ -2552,7 +2555,7 @@
     </row>
     <row r="45" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A45" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B45" s="14">
         <v>5</v>
@@ -2596,7 +2599,7 @@
     </row>
     <row r="46" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B46" s="14">
         <v>6</v>
@@ -2640,7 +2643,7 @@
     </row>
     <row r="47" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A47" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B47" s="14">
         <v>7</v>
@@ -2684,7 +2687,7 @@
     </row>
     <row r="48" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B48" s="14">
         <v>8</v>
@@ -2728,7 +2731,7 @@
     </row>
     <row r="49" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A49" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B49" s="14">
         <v>9</v>
@@ -2772,7 +2775,7 @@
     </row>
     <row r="50" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B50" s="14">
         <v>10</v>
@@ -2816,7 +2819,7 @@
     </row>
     <row r="51" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A51" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B51" s="14">
         <v>11</v>
@@ -2860,7 +2863,7 @@
     </row>
     <row r="52" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B52" s="14">
         <v>12</v>
@@ -2904,7 +2907,7 @@
     </row>
     <row r="53" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A53" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B53" s="14">
         <v>13</v>
@@ -2948,7 +2951,7 @@
     </row>
     <row r="54" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B54" s="14">
         <v>14</v>
@@ -2992,7 +2995,7 @@
     </row>
     <row r="55" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A55" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B55" s="14">
         <v>15</v>
@@ -3036,7 +3039,7 @@
     </row>
     <row r="56" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B56" s="14">
         <v>16</v>
@@ -3080,7 +3083,7 @@
     </row>
     <row r="57" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A57" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B57" s="14">
         <v>17</v>
@@ -3124,7 +3127,7 @@
     </row>
     <row r="58" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B58" s="14">
         <v>18</v>
@@ -3168,7 +3171,7 @@
     </row>
     <row r="59" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A59" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B59" s="14">
         <v>19</v>
@@ -3212,7 +3215,7 @@
     </row>
     <row r="60" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A60" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B60" s="14">
         <v>20</v>
@@ -3256,7 +3259,7 @@
     </row>
     <row r="61" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A61" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B61" s="14">
         <v>21</v>
@@ -3300,7 +3303,7 @@
     </row>
     <row r="62" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A62" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B62" s="14">
         <v>22</v>
@@ -3344,7 +3347,7 @@
     </row>
     <row r="63" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A63" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B63" s="14">
         <v>23</v>
@@ -3388,7 +3391,7 @@
     </row>
     <row r="64" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B64" s="14">
         <v>24</v>
@@ -3432,7 +3435,7 @@
     </row>
     <row r="65" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A65" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B65" s="14">
         <v>25</v>
@@ -3476,7 +3479,7 @@
     </row>
     <row r="66" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A66" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B66" s="14">
         <v>26</v>
@@ -3520,7 +3523,7 @@
     </row>
     <row r="67" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A67" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B67" s="14">
         <v>27</v>
@@ -3564,7 +3567,7 @@
     </row>
     <row r="68" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A68" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B68" s="14">
         <v>28</v>
@@ -3608,7 +3611,7 @@
     </row>
     <row r="69" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A69" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B69" s="14">
         <v>29</v>
@@ -3652,7 +3655,7 @@
     </row>
     <row r="70" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A70" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B70" s="14">
         <v>30</v>
@@ -3696,7 +3699,7 @@
     </row>
     <row r="71" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A71" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B71" s="14">
         <v>31</v>
@@ -3740,7 +3743,7 @@
     </row>
     <row r="72" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A72" s="13" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B72" s="14">
         <v>1</v>
@@ -3784,7 +3787,7 @@
     </row>
     <row r="73" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A73" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B73" s="14">
         <v>2</v>
@@ -3828,7 +3831,7 @@
     </row>
     <row r="74" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A74" s="13" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B74" s="14">
         <v>3</v>
@@ -3872,7 +3875,7 @@
     </row>
     <row r="75" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A75" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B75" s="14">
         <v>4</v>
@@ -3916,7 +3919,7 @@
     </row>
     <row r="76" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A76" s="13" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B76" s="14">
         <v>5</v>
@@ -3960,7 +3963,7 @@
     </row>
     <row r="77" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A77" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B77" s="14">
         <v>6</v>
@@ -4004,7 +4007,7 @@
     </row>
     <row r="78" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A78" s="13" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B78" s="14">
         <v>7</v>
@@ -4048,7 +4051,7 @@
     </row>
     <row r="79" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A79" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B79" s="14">
         <v>8</v>
@@ -4092,7 +4095,7 @@
     </row>
     <row r="80" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A80" s="13" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B80" s="14">
         <v>9</v>
@@ -4136,7 +4139,7 @@
     </row>
     <row r="81" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A81" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B81" s="14">
         <v>10</v>
@@ -4180,7 +4183,7 @@
     </row>
     <row r="82" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A82" s="13" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B82" s="14">
         <v>11</v>
@@ -4224,7 +4227,7 @@
     </row>
     <row r="83" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A83" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B83" s="14">
         <v>12</v>
@@ -4268,7 +4271,7 @@
     </row>
     <row r="84" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A84" s="13" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B84" s="14">
         <v>13</v>
@@ -4312,7 +4315,7 @@
     </row>
     <row r="85" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A85" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B85" s="14">
         <v>14</v>
@@ -4356,7 +4359,7 @@
     </row>
     <row r="86" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A86" s="13" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B86" s="14">
         <v>1</v>
@@ -4400,7 +4403,7 @@
     </row>
     <row r="87" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A87" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B87" s="14">
         <v>2</v>
@@ -4444,7 +4447,7 @@
     </row>
     <row r="88" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A88" s="13" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B88" s="14">
         <v>3</v>
@@ -4488,7 +4491,7 @@
     </row>
     <row r="89" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A89" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B89" s="14">
         <v>4</v>
@@ -4532,7 +4535,7 @@
     </row>
     <row r="90" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A90" s="13" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B90" s="14">
         <v>5</v>
@@ -4576,7 +4579,7 @@
     </row>
     <row r="91" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A91" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B91" s="14">
         <v>6</v>
@@ -4620,7 +4623,7 @@
     </row>
     <row r="92" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A92" s="13" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B92" s="14">
         <v>7</v>
@@ -4664,7 +4667,7 @@
     </row>
     <row r="93" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A93" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B93" s="14">
         <v>8</v>
@@ -4708,7 +4711,7 @@
     </row>
     <row r="94" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A94" s="13" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B94" s="14">
         <v>9</v>
@@ -4752,7 +4755,7 @@
     </row>
     <row r="95" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A95" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B95" s="14">
         <v>10</v>
@@ -4796,7 +4799,7 @@
     </row>
     <row r="96" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A96" s="13" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B96" s="14">
         <v>11</v>
@@ -4840,7 +4843,7 @@
     </row>
     <row r="97" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A97" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B97" s="14">
         <v>12</v>
@@ -4884,7 +4887,7 @@
     </row>
     <row r="98" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A98" s="13" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B98" s="14">
         <v>13</v>
@@ -4928,7 +4931,7 @@
     </row>
     <row r="99" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A99" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B99" s="14">
         <v>14</v>
@@ -4972,7 +4975,7 @@
     </row>
     <row r="100" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A100" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B100" s="17">
         <v>1</v>
@@ -5016,7 +5019,7 @@
     </row>
     <row r="101" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A101" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B101" s="17">
         <v>2</v>
@@ -5060,7 +5063,7 @@
     </row>
     <row r="102" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A102" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B102" s="17">
         <v>3</v>
@@ -5104,7 +5107,7 @@
     </row>
     <row r="103" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A103" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B103" s="17">
         <v>4</v>
@@ -5148,7 +5151,7 @@
     </row>
     <row r="104" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A104" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B104" s="17">
         <v>5</v>
@@ -5192,7 +5195,7 @@
     </row>
     <row r="105" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A105" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B105" s="17">
         <v>6</v>
@@ -5236,7 +5239,7 @@
     </row>
     <row r="106" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A106" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B106" s="17">
         <v>7</v>
@@ -5280,7 +5283,7 @@
     </row>
     <row r="107" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A107" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B107" s="17">
         <v>8</v>
@@ -5324,7 +5327,7 @@
     </row>
     <row r="108" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A108" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B108" s="17">
         <v>9</v>
@@ -5368,7 +5371,7 @@
     </row>
     <row r="109" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A109" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B109" s="17">
         <v>10</v>
@@ -5412,7 +5415,7 @@
     </row>
     <row r="110" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A110" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B110" s="17">
         <v>11</v>
@@ -5456,7 +5459,7 @@
     </row>
     <row r="111" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A111" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B111" s="17">
         <v>12</v>
@@ -5500,7 +5503,7 @@
     </row>
     <row r="112" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A112" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B112" s="17">
         <v>13</v>
@@ -5544,7 +5547,7 @@
     </row>
     <row r="113" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A113" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B113" s="17">
         <v>14</v>
@@ -5588,7 +5591,7 @@
     </row>
     <row r="114" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A114" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B114" s="17">
         <v>15</v>
@@ -5632,7 +5635,7 @@
     </row>
     <row r="115" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A115" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B115" s="17">
         <v>16</v>
@@ -5676,7 +5679,7 @@
     </row>
     <row r="116" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A116" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B116" s="17">
         <v>17</v>
@@ -5720,7 +5723,7 @@
     </row>
     <row r="117" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A117" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B117" s="17">
         <v>18</v>
@@ -5764,7 +5767,7 @@
     </row>
     <row r="118" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A118" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B118" s="17">
         <v>19</v>
@@ -5808,7 +5811,7 @@
     </row>
     <row r="119" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A119" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B119" s="17">
         <v>20</v>
@@ -5852,7 +5855,7 @@
     </row>
     <row r="120" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A120" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B120" s="23">
         <v>1</v>
@@ -5896,7 +5899,7 @@
     </row>
     <row r="121" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A121" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B121" s="24">
         <v>2</v>
@@ -5940,7 +5943,7 @@
     </row>
     <row r="122" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A122" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B122" s="23">
         <v>3</v>
@@ -5984,7 +5987,7 @@
     </row>
     <row r="123" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A123" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B123" s="24">
         <v>4</v>
@@ -6028,7 +6031,7 @@
     </row>
     <row r="124" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A124" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B124" s="23">
         <v>5</v>
@@ -6072,7 +6075,7 @@
     </row>
     <row r="125" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A125" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B125" s="24">
         <v>6</v>
@@ -6116,7 +6119,7 @@
     </row>
     <row r="126" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A126" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B126" s="23">
         <v>7</v>
@@ -6160,7 +6163,7 @@
     </row>
     <row r="127" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A127" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B127" s="24">
         <v>8</v>
@@ -6204,7 +6207,7 @@
     </row>
     <row r="128" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A128" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B128" s="23">
         <v>9</v>
@@ -6248,7 +6251,7 @@
     </row>
     <row r="129" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A129" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B129" s="24">
         <v>10</v>
@@ -6292,7 +6295,7 @@
     </row>
     <row r="130" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A130" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B130" s="23">
         <v>11</v>
@@ -6336,7 +6339,7 @@
     </row>
     <row r="131" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A131" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B131" s="24">
         <v>12</v>
@@ -6380,7 +6383,7 @@
     </row>
     <row r="132" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A132" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B132" s="23">
         <v>13</v>
@@ -6424,7 +6427,7 @@
     </row>
     <row r="133" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A133" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B133" s="24">
         <v>14</v>
@@ -6468,7 +6471,7 @@
     </row>
     <row r="134" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A134" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B134" s="23">
         <v>15</v>
@@ -19520,7 +19523,7 @@
   <sheetData>
     <row r="1" ht="18" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="4">
@@ -21278,7 +21281,7 @@
     </row>
     <row r="41" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A41" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B41" s="14">
         <v>1</v>
@@ -21322,7 +21325,7 @@
     </row>
     <row r="42" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B42" s="14">
         <v>2</v>
@@ -21366,7 +21369,7 @@
     </row>
     <row r="43" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A43" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B43" s="14">
         <v>3</v>
@@ -21410,7 +21413,7 @@
     </row>
     <row r="44" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B44" s="14">
         <v>4</v>
@@ -21454,7 +21457,7 @@
     </row>
     <row r="45" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A45" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B45" s="14">
         <v>5</v>
@@ -21498,7 +21501,7 @@
     </row>
     <row r="46" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B46" s="14">
         <v>6</v>
@@ -21542,7 +21545,7 @@
     </row>
     <row r="47" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A47" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B47" s="14">
         <v>7</v>
@@ -21586,7 +21589,7 @@
     </row>
     <row r="48" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B48" s="14">
         <v>8</v>
@@ -21630,7 +21633,7 @@
     </row>
     <row r="49" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A49" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B49" s="14">
         <v>9</v>
@@ -21674,7 +21677,7 @@
     </row>
     <row r="50" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B50" s="14">
         <v>10</v>
@@ -21718,7 +21721,7 @@
     </row>
     <row r="51" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A51" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B51" s="14">
         <v>11</v>
@@ -21762,7 +21765,7 @@
     </row>
     <row r="52" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B52" s="14">
         <v>12</v>
@@ -21806,7 +21809,7 @@
     </row>
     <row r="53" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A53" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B53" s="14">
         <v>13</v>
@@ -21850,7 +21853,7 @@
     </row>
     <row r="54" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B54" s="14">
         <v>14</v>
@@ -21894,7 +21897,7 @@
     </row>
     <row r="55" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A55" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B55" s="14">
         <v>15</v>
@@ -21938,7 +21941,7 @@
     </row>
     <row r="56" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B56" s="14">
         <v>16</v>
@@ -21982,7 +21985,7 @@
     </row>
     <row r="57" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A57" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B57" s="14">
         <v>17</v>
@@ -22026,7 +22029,7 @@
     </row>
     <row r="58" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B58" s="14">
         <v>18</v>
@@ -22070,7 +22073,7 @@
     </row>
     <row r="59" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A59" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B59" s="14">
         <v>19</v>
@@ -22114,7 +22117,7 @@
     </row>
     <row r="60" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A60" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B60" s="14">
         <v>20</v>
@@ -22158,7 +22161,7 @@
     </row>
     <row r="61" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A61" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B61" s="14">
         <v>21</v>
@@ -22202,7 +22205,7 @@
     </row>
     <row r="62" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A62" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B62" s="14">
         <v>22</v>
@@ -22246,7 +22249,7 @@
     </row>
     <row r="63" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A63" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B63" s="14">
         <v>23</v>
@@ -22290,7 +22293,7 @@
     </row>
     <row r="64" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B64" s="14">
         <v>24</v>
@@ -22334,7 +22337,7 @@
     </row>
     <row r="65" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A65" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B65" s="14">
         <v>25</v>
@@ -22378,7 +22381,7 @@
     </row>
     <row r="66" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A66" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B66" s="14">
         <v>26</v>
@@ -22422,7 +22425,7 @@
     </row>
     <row r="67" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A67" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B67" s="14">
         <v>27</v>
@@ -22466,7 +22469,7 @@
     </row>
     <row r="68" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A68" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B68" s="14">
         <v>28</v>
@@ -22510,7 +22513,7 @@
     </row>
     <row r="69" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A69" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B69" s="14">
         <v>29</v>
@@ -22554,7 +22557,7 @@
     </row>
     <row r="70" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A70" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B70" s="14">
         <v>30</v>
@@ -22598,7 +22601,7 @@
     </row>
     <row r="71" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A71" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B71" s="14">
         <v>31</v>
@@ -22642,7 +22645,7 @@
     </row>
     <row r="72" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A72" s="13" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B72" s="14">
         <v>1</v>
@@ -22686,7 +22689,7 @@
     </row>
     <row r="73" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A73" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B73" s="14">
         <v>2</v>
@@ -22730,7 +22733,7 @@
     </row>
     <row r="74" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A74" s="13" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B74" s="14">
         <v>3</v>
@@ -22774,7 +22777,7 @@
     </row>
     <row r="75" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A75" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B75" s="14">
         <v>4</v>
@@ -22818,7 +22821,7 @@
     </row>
     <row r="76" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A76" s="13" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B76" s="14">
         <v>5</v>
@@ -22862,7 +22865,7 @@
     </row>
     <row r="77" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A77" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B77" s="14">
         <v>6</v>
@@ -22906,7 +22909,7 @@
     </row>
     <row r="78" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A78" s="13" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B78" s="14">
         <v>7</v>
@@ -22950,7 +22953,7 @@
     </row>
     <row r="79" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A79" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B79" s="14">
         <v>8</v>
@@ -22994,7 +22997,7 @@
     </row>
     <row r="80" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A80" s="13" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B80" s="14">
         <v>9</v>
@@ -23038,7 +23041,7 @@
     </row>
     <row r="81" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A81" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B81" s="14">
         <v>10</v>
@@ -23082,7 +23085,7 @@
     </row>
     <row r="82" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A82" s="13" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B82" s="14">
         <v>11</v>
@@ -23126,7 +23129,7 @@
     </row>
     <row r="83" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A83" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B83" s="14">
         <v>12</v>
@@ -23170,7 +23173,7 @@
     </row>
     <row r="84" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A84" s="13" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B84" s="14">
         <v>13</v>
@@ -23214,7 +23217,7 @@
     </row>
     <row r="85" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A85" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B85" s="14">
         <v>14</v>
@@ -23258,7 +23261,7 @@
     </row>
     <row r="86" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A86" s="13" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B86" s="14">
         <v>1</v>
@@ -23302,7 +23305,7 @@
     </row>
     <row r="87" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A87" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B87" s="14">
         <v>2</v>
@@ -23346,7 +23349,7 @@
     </row>
     <row r="88" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A88" s="13" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B88" s="14">
         <v>3</v>
@@ -23390,7 +23393,7 @@
     </row>
     <row r="89" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A89" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B89" s="14">
         <v>4</v>
@@ -23434,7 +23437,7 @@
     </row>
     <row r="90" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A90" s="13" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B90" s="14">
         <v>5</v>
@@ -23478,7 +23481,7 @@
     </row>
     <row r="91" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A91" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B91" s="14">
         <v>6</v>
@@ -23522,7 +23525,7 @@
     </row>
     <row r="92" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A92" s="13" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B92" s="14">
         <v>7</v>
@@ -23566,7 +23569,7 @@
     </row>
     <row r="93" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A93" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B93" s="14">
         <v>8</v>
@@ -23610,7 +23613,7 @@
     </row>
     <row r="94" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A94" s="13" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B94" s="14">
         <v>9</v>
@@ -23654,7 +23657,7 @@
     </row>
     <row r="95" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A95" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B95" s="14">
         <v>10</v>
@@ -23698,7 +23701,7 @@
     </row>
     <row r="96" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A96" s="13" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B96" s="14">
         <v>11</v>
@@ -23742,7 +23745,7 @@
     </row>
     <row r="97" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A97" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B97" s="14">
         <v>12</v>
@@ -23786,7 +23789,7 @@
     </row>
     <row r="98" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A98" s="13" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B98" s="14">
         <v>13</v>
@@ -23830,7 +23833,7 @@
     </row>
     <row r="99" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A99" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B99" s="14">
         <v>14</v>
@@ -23874,7 +23877,7 @@
     </row>
     <row r="100" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A100" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B100" s="17">
         <v>1</v>
@@ -23918,7 +23921,7 @@
     </row>
     <row r="101" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A101" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B101" s="17">
         <v>2</v>
@@ -23962,7 +23965,7 @@
     </row>
     <row r="102" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A102" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B102" s="17">
         <v>3</v>
@@ -24006,7 +24009,7 @@
     </row>
     <row r="103" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A103" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B103" s="17">
         <v>4</v>
@@ -24050,7 +24053,7 @@
     </row>
     <row r="104" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A104" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B104" s="17">
         <v>5</v>
@@ -24094,7 +24097,7 @@
     </row>
     <row r="105" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A105" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B105" s="17">
         <v>6</v>
@@ -24138,7 +24141,7 @@
     </row>
     <row r="106" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A106" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B106" s="17">
         <v>7</v>
@@ -24182,7 +24185,7 @@
     </row>
     <row r="107" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A107" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B107" s="17">
         <v>8</v>
@@ -24226,7 +24229,7 @@
     </row>
     <row r="108" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A108" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B108" s="17">
         <v>9</v>
@@ -24270,7 +24273,7 @@
     </row>
     <row r="109" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A109" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B109" s="17">
         <v>10</v>
@@ -24314,7 +24317,7 @@
     </row>
     <row r="110" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A110" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B110" s="17">
         <v>11</v>
@@ -24358,7 +24361,7 @@
     </row>
     <row r="111" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A111" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B111" s="17">
         <v>12</v>
@@ -24402,7 +24405,7 @@
     </row>
     <row r="112" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A112" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B112" s="17">
         <v>13</v>
@@ -24446,7 +24449,7 @@
     </row>
     <row r="113" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A113" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B113" s="17">
         <v>14</v>
@@ -24490,7 +24493,7 @@
     </row>
     <row r="114" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A114" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B114" s="17">
         <v>15</v>
@@ -24534,7 +24537,7 @@
     </row>
     <row r="115" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A115" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B115" s="17">
         <v>16</v>
@@ -24578,7 +24581,7 @@
     </row>
     <row r="116" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A116" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B116" s="17">
         <v>17</v>
@@ -24622,7 +24625,7 @@
     </row>
     <row r="117" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A117" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B117" s="17">
         <v>18</v>
@@ -24666,7 +24669,7 @@
     </row>
     <row r="118" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A118" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B118" s="17">
         <v>19</v>
@@ -24710,7 +24713,7 @@
     </row>
     <row r="119" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A119" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B119" s="17">
         <v>20</v>
@@ -24754,7 +24757,7 @@
     </row>
     <row r="120" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A120" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B120" s="23">
         <v>1</v>
@@ -24798,7 +24801,7 @@
     </row>
     <row r="121" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A121" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B121" s="24">
         <v>2</v>
@@ -24842,7 +24845,7 @@
     </row>
     <row r="122" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A122" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B122" s="23">
         <v>3</v>
@@ -24886,7 +24889,7 @@
     </row>
     <row r="123" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A123" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B123" s="24">
         <v>4</v>
@@ -24930,7 +24933,7 @@
     </row>
     <row r="124" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A124" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B124" s="23">
         <v>5</v>
@@ -24974,7 +24977,7 @@
     </row>
     <row r="125" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A125" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B125" s="24">
         <v>6</v>
@@ -25018,7 +25021,7 @@
     </row>
     <row r="126" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A126" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B126" s="23">
         <v>7</v>
@@ -25062,7 +25065,7 @@
     </row>
     <row r="127" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A127" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B127" s="24">
         <v>8</v>
@@ -25106,7 +25109,7 @@
     </row>
     <row r="128" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A128" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B128" s="23">
         <v>9</v>
@@ -25150,7 +25153,7 @@
     </row>
     <row r="129" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A129" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B129" s="24">
         <v>10</v>
@@ -25194,7 +25197,7 @@
     </row>
     <row r="130" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A130" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B130" s="23">
         <v>11</v>
@@ -25238,7 +25241,7 @@
     </row>
     <row r="131" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A131" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B131" s="24">
         <v>12</v>
@@ -25282,7 +25285,7 @@
     </row>
     <row r="132" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A132" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B132" s="23">
         <v>13</v>
@@ -25326,7 +25329,7 @@
     </row>
     <row r="133" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A133" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B133" s="24">
         <v>14</v>
@@ -25370,7 +25373,7 @@
     </row>
     <row r="134" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A134" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B134" s="23">
         <v>15</v>

</xml_diff>